<commit_message>
Update notebook doc links, dump_path, observation process cleanup
- Notebook links point to xspatula_core_docs and the new
  /observation/ doc pages (cells 3.2.1, 3.2.6-3.2.9)
- Add dump_path to the setup scheme file
- Remove measurement process files and old agrolab insert files

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ai4sh/import_data/utility/observation/excel/preparation.xlsx
+++ b/ai4sh/import_data/utility/observation/excel/preparation.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="130">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -70,6 +70,15 @@
     <t xml:space="preserve">Owen drying before analysis</t>
   </si>
   <si>
+    <t xml:space="preserve">sieving&lt;4mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">s4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sieving to fraction &lt; 4 mm</t>
+  </si>
+  <si>
     <t xml:space="preserve">drying and sieving&lt;2mm</t>
   </si>
   <si>
@@ -347,6 +356,15 @@
   </si>
   <si>
     <t xml:space="preserve">Manual selection of aggregates from sample with mixed grains and aggregates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dired aggregate selection</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dagg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manual selection of dired aggregates from sample with mixed grains and aggregates</t>
   </si>
   <si>
     <t xml:space="preserve">grain selection</t>
@@ -602,7 +620,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36.25"/>
@@ -738,98 +756,98 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="1" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="D11" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="1" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="1" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
+      <c r="B14" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>52</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>54</v>
@@ -1155,6 +1173,34 @@
       </c>
       <c r="D39" s="1" t="s">
         <v>123</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>